<commit_message>
Task O done on Simulation, needs to be tested next lab
</commit_message>
<xml_diff>
--- a/UR5 Tasks.xlsx
+++ b/UR5 Tasks.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ucliveac-my.sharepoint.com/personal/mcu55_uclive_ac_nz/Documents/4th Year/ENMT482/Assignment 2/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ucliveac-my.sharepoint.com/personal/mcu55_uclive_ac_nz/Documents/4th Year/ENMT482/ENMT482-Robot-Coffee-Special/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="141" documentId="8_{5F62A8B3-761C-4507-BA16-EE4921CCE146}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5AE1458C-C527-448C-A7EF-2A0F88453AF1}"/>
+  <xr:revisionPtr revIDLastSave="163" documentId="8_{5F62A8B3-761C-4507-BA16-EE4921CCE146}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7B0EBB06-80A5-4437-96C0-6BD21D058AD3}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="64">
   <si>
     <t>ACTION ITEMS</t>
   </si>
@@ -397,7 +397,7 @@
     </xf>
     <xf numFmtId="9" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -438,9 +438,6 @@
     </xf>
     <xf numFmtId="9" fontId="7" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
@@ -496,7 +493,12 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="39">
+  <dxfs count="23">
+    <dxf>
+      <font>
+        <color theme="0" tint="-0.499984740745262"/>
+      </font>
+    </dxf>
     <dxf>
       <font>
         <color theme="0" tint="-0.499984740745262"/>
@@ -531,151 +533,6 @@
           <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0" tint="-0.499984740745262"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0" tint="-0.499984740745262"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0" tint="-0.499984740745262"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0" tint="-0.499984740745262"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0" tint="-0.499984740745262"/>
-      </font>
     </dxf>
     <dxf>
       <font>
@@ -892,15 +749,15 @@
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="ToDoList" pivot="0" count="9" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
-      <tableStyleElement type="wholeTable" dxfId="38"/>
-      <tableStyleElement type="headerRow" dxfId="37"/>
-      <tableStyleElement type="totalRow" dxfId="36"/>
-      <tableStyleElement type="firstColumn" dxfId="35"/>
-      <tableStyleElement type="lastColumn" dxfId="34"/>
-      <tableStyleElement type="firstRowStripe" dxfId="33"/>
-      <tableStyleElement type="secondRowStripe" dxfId="32"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="31"/>
-      <tableStyleElement type="secondColumnStripe" dxfId="30"/>
+      <tableStyleElement type="wholeTable" dxfId="22"/>
+      <tableStyleElement type="headerRow" dxfId="21"/>
+      <tableStyleElement type="totalRow" dxfId="20"/>
+      <tableStyleElement type="firstColumn" dxfId="19"/>
+      <tableStyleElement type="lastColumn" dxfId="18"/>
+      <tableStyleElement type="firstRowStripe" dxfId="17"/>
+      <tableStyleElement type="secondRowStripe" dxfId="16"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="15"/>
+      <tableStyleElement type="secondColumnStripe" dxfId="14"/>
     </tableStyle>
   </tableStyles>
   <colors>
@@ -920,19 +777,19 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table137" displayName="Table137" ref="B4:H31" totalsRowShown="0" headerRowDxfId="29" dataDxfId="28">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table137" displayName="Table137" ref="B4:H31" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
   <autoFilter ref="B4:H31" xr:uid="{00000000-0009-0000-0100-000006000000}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B5:H31">
     <sortCondition descending="1" ref="E4:E31"/>
   </sortState>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="ACTION ITEM" dataDxfId="27"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Task" dataDxfId="26"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="OWNER" dataDxfId="25"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="DUE" dataDxfId="24"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="DONE" dataDxfId="23"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="STATUS" dataDxfId="22"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="NOTES" dataDxfId="21"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="ACTION ITEM" dataDxfId="11"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Task" dataDxfId="10"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="OWNER" dataDxfId="9"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="DUE" dataDxfId="8"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="DONE" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="STATUS" dataDxfId="6"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="NOTES" dataDxfId="5"/>
   </tableColumns>
   <tableStyleInfo name="ToDoList" showFirstColumn="1" showLastColumn="0" showRowStripes="1" showColumnStripes="1"/>
 </table>
@@ -1233,19 +1090,19 @@
       <c r="I1" s="2"/>
     </row>
     <row r="2" spans="2:11" s="7" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B2" s="23" t="s">
+      <c r="B2" s="22" t="s">
         <v>60</v>
       </c>
-      <c r="D2" s="21" t="s">
+      <c r="D2" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="20">
+      <c r="E2" s="19">
         <v>46278</v>
       </c>
-      <c r="G2" s="21" t="s">
+      <c r="G2" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="H2" s="22">
+      <c r="H2" s="21">
         <v>46182.479166666664</v>
       </c>
       <c r="K2" s="10"/>
@@ -1259,7 +1116,7 @@
       <c r="B4" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="19" t="s">
+      <c r="C4" s="18" t="s">
         <v>14</v>
       </c>
       <c r="D4" s="5" t="s">
@@ -1268,10 +1125,10 @@
       <c r="E4" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="F4" s="17" t="s">
+      <c r="F4" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="G4" s="18" t="s">
+      <c r="G4" s="17" t="s">
         <v>7</v>
       </c>
       <c r="H4" s="5" t="s">
@@ -1279,36 +1136,38 @@
       </c>
     </row>
     <row r="5" spans="2:11" ht="40" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B5" s="28" t="s">
+      <c r="B5" s="27" t="s">
         <v>38</v>
       </c>
-      <c r="C5" s="31" t="s">
+      <c r="C5" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="3"/>
+      <c r="D5" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="E5" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="F5" s="24"/>
+      <c r="F5" s="23"/>
       <c r="G5" s="13" t="s">
         <v>10</v>
       </c>
       <c r="H5" s="4"/>
     </row>
     <row r="6" spans="2:11" s="7" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B6" s="28" t="s">
+      <c r="B6" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="C6" s="31" t="s">
+      <c r="C6" s="30" t="s">
         <v>15</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E6" s="29" t="s">
+      <c r="E6" s="28" t="s">
         <v>61</v>
       </c>
-      <c r="F6" s="24" t="s">
+      <c r="F6" s="23" t="s">
         <v>12</v>
       </c>
       <c r="G6" s="14" t="s">
@@ -1318,17 +1177,19 @@
       <c r="J6" s="10"/>
     </row>
     <row r="7" spans="2:11" s="7" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B7" s="28" t="s">
+      <c r="B7" s="27" t="s">
         <v>40</v>
       </c>
-      <c r="C7" s="31" t="s">
+      <c r="C7" s="30" t="s">
         <v>18</v>
       </c>
-      <c r="D7" s="3"/>
-      <c r="E7" s="30" t="s">
+      <c r="D7" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E7" s="29" t="s">
         <v>61</v>
       </c>
-      <c r="F7" s="24"/>
+      <c r="F7" s="23"/>
       <c r="G7" s="13" t="s">
         <v>10</v>
       </c>
@@ -1336,17 +1197,19 @@
       <c r="J7" s="10"/>
     </row>
     <row r="8" spans="2:11" s="7" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B8" s="28" t="s">
+      <c r="B8" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="C8" s="31" t="s">
+      <c r="C8" s="30" t="s">
         <v>19</v>
       </c>
-      <c r="D8" s="3"/>
+      <c r="D8" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="E8" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="F8" s="24"/>
+      <c r="F8" s="23"/>
       <c r="G8" s="13" t="s">
         <v>10</v>
       </c>
@@ -1354,44 +1217,48 @@
       <c r="J8" s="10"/>
     </row>
     <row r="9" spans="2:11" s="7" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B9" s="28" t="s">
+      <c r="B9" s="27" t="s">
         <v>42</v>
       </c>
-      <c r="C9" s="31" t="s">
+      <c r="C9" s="30" t="s">
         <v>20</v>
       </c>
-      <c r="D9" s="3"/>
+      <c r="D9" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="E9" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="F9" s="24"/>
+      <c r="F9" s="23"/>
       <c r="G9" s="13" t="s">
         <v>10</v>
       </c>
       <c r="H9" s="4"/>
     </row>
     <row r="10" spans="2:11" s="7" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B10" s="28" t="s">
+      <c r="B10" s="27" t="s">
         <v>43</v>
       </c>
-      <c r="C10" s="31" t="s">
+      <c r="C10" s="30" t="s">
         <v>21</v>
       </c>
-      <c r="D10" s="3"/>
+      <c r="D10" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="E10" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="F10" s="24"/>
+      <c r="F10" s="23"/>
       <c r="G10" s="13" t="s">
         <v>10</v>
       </c>
       <c r="H10" s="4"/>
     </row>
     <row r="11" spans="2:11" s="7" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B11" s="28" t="s">
+      <c r="B11" s="27" t="s">
         <v>44</v>
       </c>
-      <c r="C11" s="31" t="s">
+      <c r="C11" s="30" t="s">
         <v>22</v>
       </c>
       <c r="D11" s="3" t="s">
@@ -1400,262 +1267,292 @@
       <c r="E11" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="F11" s="24"/>
+      <c r="F11" s="23"/>
       <c r="G11" s="13" t="s">
         <v>10</v>
       </c>
       <c r="H11" s="4"/>
     </row>
     <row r="12" spans="2:11" s="7" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B12" s="28" t="s">
+      <c r="B12" s="27" t="s">
         <v>45</v>
       </c>
-      <c r="C12" s="31" t="s">
+      <c r="C12" s="30" t="s">
         <v>23</v>
       </c>
-      <c r="D12" s="3"/>
+      <c r="D12" s="3" t="s">
+        <v>16</v>
+      </c>
       <c r="E12" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="F12" s="24"/>
+      <c r="F12" s="23"/>
       <c r="G12" s="13" t="s">
         <v>10</v>
       </c>
       <c r="H12" s="4"/>
     </row>
     <row r="13" spans="2:11" s="7" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B13" s="28" t="s">
+      <c r="B13" s="27" t="s">
         <v>46</v>
       </c>
-      <c r="C13" s="31" t="s">
+      <c r="C13" s="30" t="s">
         <v>24</v>
       </c>
-      <c r="D13" s="3"/>
+      <c r="D13" s="3" t="s">
+        <v>16</v>
+      </c>
       <c r="E13" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="F13" s="24"/>
+      <c r="F13" s="23"/>
       <c r="G13" s="13" t="s">
         <v>10</v>
       </c>
       <c r="H13" s="4"/>
     </row>
     <row r="14" spans="2:11" s="7" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B14" s="28" t="s">
+      <c r="B14" s="27" t="s">
         <v>47</v>
       </c>
-      <c r="C14" s="31" t="s">
+      <c r="C14" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="D14" s="3"/>
+      <c r="D14" s="3" t="s">
+        <v>16</v>
+      </c>
       <c r="E14" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="F14" s="24"/>
+      <c r="F14" s="23"/>
       <c r="G14" s="13" t="s">
         <v>10</v>
       </c>
       <c r="H14" s="4"/>
     </row>
     <row r="15" spans="2:11" s="7" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B15" s="28" t="s">
+      <c r="B15" s="27" t="s">
         <v>48</v>
       </c>
-      <c r="C15" s="31" t="s">
+      <c r="C15" s="30" t="s">
         <v>26</v>
       </c>
-      <c r="D15" s="3"/>
+      <c r="D15" s="3" t="s">
+        <v>16</v>
+      </c>
       <c r="E15" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="F15" s="24"/>
+      <c r="F15" s="23"/>
       <c r="G15" s="13" t="s">
         <v>10</v>
       </c>
       <c r="H15" s="4"/>
     </row>
     <row r="16" spans="2:11" s="7" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B16" s="28" t="s">
+      <c r="B16" s="27" t="s">
         <v>49</v>
       </c>
-      <c r="C16" s="31" t="s">
+      <c r="C16" s="30" t="s">
         <v>27</v>
       </c>
-      <c r="D16" s="3"/>
+      <c r="D16" s="3" t="s">
+        <v>16</v>
+      </c>
       <c r="E16" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="F16" s="24"/>
+      <c r="F16" s="23"/>
       <c r="G16" s="14" t="s">
         <v>10</v>
       </c>
       <c r="H16" s="4"/>
     </row>
     <row r="17" spans="2:10" s="7" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B17" s="28" t="s">
+      <c r="B17" s="27" t="s">
         <v>50</v>
       </c>
-      <c r="C17" s="31" t="s">
+      <c r="C17" s="30" t="s">
         <v>28</v>
       </c>
-      <c r="D17" s="3"/>
-      <c r="E17" s="29" t="s">
+      <c r="D17" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E17" s="28" t="s">
         <v>61</v>
       </c>
-      <c r="F17" s="24"/>
+      <c r="F17" s="23"/>
       <c r="G17" s="14" t="s">
         <v>10</v>
       </c>
       <c r="H17" s="4"/>
     </row>
     <row r="18" spans="2:10" s="7" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B18" s="28" t="s">
+      <c r="B18" s="27" t="s">
         <v>51</v>
       </c>
-      <c r="C18" s="31" t="s">
+      <c r="C18" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="D18" s="3"/>
+      <c r="D18" s="3" t="s">
+        <v>16</v>
+      </c>
       <c r="E18" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="F18" s="24"/>
+      <c r="F18" s="23"/>
       <c r="G18" s="14" t="s">
         <v>10</v>
       </c>
       <c r="H18" s="4"/>
     </row>
     <row r="19" spans="2:10" s="7" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B19" s="28" t="s">
+      <c r="B19" s="27" t="s">
         <v>52</v>
       </c>
-      <c r="C19" s="31" t="s">
+      <c r="C19" s="30" t="s">
         <v>30</v>
       </c>
-      <c r="D19" s="3"/>
+      <c r="D19" s="3" t="s">
+        <v>9</v>
+      </c>
       <c r="E19" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="F19" s="24"/>
-      <c r="G19" s="14" t="s">
-        <v>10</v>
+      <c r="F19" s="23"/>
+      <c r="G19" s="14">
+        <v>0.5</v>
       </c>
       <c r="H19" s="4"/>
     </row>
     <row r="20" spans="2:10" s="7" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B20" s="28" t="s">
+      <c r="B20" s="27" t="s">
         <v>53</v>
       </c>
-      <c r="C20" s="31" t="s">
+      <c r="C20" s="30" t="s">
         <v>31</v>
       </c>
-      <c r="D20" s="3"/>
+      <c r="D20" s="3" t="s">
+        <v>9</v>
+      </c>
       <c r="E20" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="F20" s="24"/>
+      <c r="F20" s="23"/>
       <c r="G20" s="14" t="s">
         <v>10</v>
       </c>
       <c r="H20" s="4"/>
     </row>
     <row r="21" spans="2:10" s="7" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B21" s="28" t="s">
+      <c r="B21" s="27" t="s">
         <v>54</v>
       </c>
-      <c r="C21" s="31" t="s">
+      <c r="C21" s="30" t="s">
         <v>32</v>
       </c>
-      <c r="D21" s="3"/>
+      <c r="D21" s="3" t="s">
+        <v>9</v>
+      </c>
       <c r="E21" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="F21" s="24"/>
+      <c r="F21" s="23"/>
       <c r="G21" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="H21" s="16"/>
+      <c r="H21" s="15"/>
     </row>
     <row r="22" spans="2:10" s="7" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B22" s="28" t="s">
+      <c r="B22" s="27" t="s">
         <v>55</v>
       </c>
-      <c r="C22" s="31" t="s">
+      <c r="C22" s="30" t="s">
         <v>33</v>
       </c>
-      <c r="D22" s="3"/>
+      <c r="D22" s="3" t="s">
+        <v>9</v>
+      </c>
       <c r="E22" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="F22" s="24"/>
+      <c r="F22" s="23"/>
       <c r="G22" s="14" t="s">
         <v>10</v>
       </c>
       <c r="H22" s="4"/>
     </row>
     <row r="23" spans="2:10" s="7" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B23" s="28" t="s">
+      <c r="B23" s="27" t="s">
         <v>56</v>
       </c>
-      <c r="C23" s="31" t="s">
+      <c r="C23" s="30" t="s">
         <v>34</v>
       </c>
-      <c r="D23" s="3"/>
+      <c r="D23" s="3" t="s">
+        <v>9</v>
+      </c>
       <c r="E23" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="F23" s="24"/>
+      <c r="F23" s="23"/>
       <c r="G23" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="H23" s="16"/>
+      <c r="H23" s="15"/>
     </row>
     <row r="24" spans="2:10" s="7" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B24" s="28" t="s">
+      <c r="B24" s="27" t="s">
         <v>57</v>
       </c>
-      <c r="C24" s="31" t="s">
+      <c r="C24" s="30" t="s">
         <v>35</v>
       </c>
-      <c r="D24" s="15"/>
+      <c r="D24" s="3" t="s">
+        <v>9</v>
+      </c>
       <c r="E24" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="F24" s="24"/>
+      <c r="F24" s="23"/>
       <c r="G24" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="H24" s="16"/>
+      <c r="H24" s="15"/>
     </row>
     <row r="25" spans="2:10" s="7" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B25" s="28" t="s">
+      <c r="B25" s="27" t="s">
         <v>58</v>
       </c>
-      <c r="C25" s="31" t="s">
+      <c r="C25" s="30" t="s">
         <v>36</v>
       </c>
-      <c r="D25" s="15"/>
+      <c r="D25" s="3" t="s">
+        <v>9</v>
+      </c>
       <c r="E25" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="F25" s="24"/>
+      <c r="F25" s="23"/>
       <c r="G25" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="H25" s="16"/>
+      <c r="H25" s="15"/>
     </row>
     <row r="26" spans="2:10" s="7" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B26" s="28" t="s">
+      <c r="B26" s="27" t="s">
         <v>59</v>
       </c>
-      <c r="C26" s="31" t="s">
+      <c r="C26" s="30" t="s">
         <v>37</v>
       </c>
-      <c r="D26" s="16"/>
+      <c r="D26" s="3" t="s">
+        <v>9</v>
+      </c>
       <c r="E26" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="F26" s="26"/>
+      <c r="F26" s="25"/>
       <c r="G26" s="14" t="s">
         <v>10</v>
       </c>
@@ -1664,65 +1561,68 @@
     </row>
     <row r="27" spans="2:10" s="7" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B27" s="3"/>
-      <c r="C27" s="16"/>
-      <c r="D27" s="16"/>
-      <c r="E27" s="25"/>
-      <c r="F27" s="26"/>
-      <c r="G27" s="27"/>
+      <c r="C27" s="15"/>
+      <c r="D27" s="15"/>
+      <c r="E27" s="24"/>
+      <c r="F27" s="25"/>
+      <c r="G27" s="26"/>
       <c r="H27" s="4"/>
       <c r="J27"/>
     </row>
     <row r="28" spans="2:10" ht="14.1" x14ac:dyDescent="0.45">
       <c r="B28" s="3"/>
-      <c r="C28" s="16"/>
-      <c r="D28" s="16"/>
-      <c r="E28" s="25"/>
-      <c r="F28" s="26"/>
-      <c r="G28" s="27"/>
+      <c r="C28" s="15"/>
+      <c r="D28" s="15"/>
+      <c r="E28" s="24"/>
+      <c r="F28" s="25"/>
+      <c r="G28" s="26"/>
       <c r="H28" s="4"/>
     </row>
     <row r="29" spans="2:10" ht="14.1" x14ac:dyDescent="0.45">
       <c r="B29" s="3"/>
-      <c r="C29" s="16"/>
-      <c r="D29" s="16"/>
-      <c r="E29" s="25"/>
-      <c r="F29" s="26"/>
-      <c r="G29" s="27"/>
+      <c r="C29" s="15"/>
+      <c r="D29" s="15"/>
+      <c r="E29" s="24"/>
+      <c r="F29" s="25"/>
+      <c r="G29" s="26"/>
       <c r="H29" s="4"/>
     </row>
     <row r="30" spans="2:10" ht="14.1" x14ac:dyDescent="0.45">
       <c r="B30" s="3"/>
-      <c r="C30" s="16"/>
-      <c r="D30" s="16"/>
-      <c r="E30" s="25"/>
-      <c r="F30" s="26"/>
-      <c r="G30" s="27"/>
+      <c r="C30" s="15"/>
+      <c r="D30" s="15"/>
+      <c r="E30" s="24"/>
+      <c r="F30" s="25"/>
+      <c r="G30" s="26"/>
       <c r="H30" s="4"/>
     </row>
     <row r="31" spans="2:10" ht="14.1" x14ac:dyDescent="0.45">
       <c r="B31" s="3"/>
-      <c r="C31" s="16"/>
-      <c r="D31" s="16"/>
-      <c r="E31" s="25"/>
-      <c r="F31" s="26"/>
-      <c r="G31" s="27"/>
+      <c r="C31" s="15"/>
+      <c r="D31" s="15"/>
+      <c r="E31" s="24"/>
+      <c r="F31" s="25"/>
+      <c r="G31" s="26"/>
       <c r="H31" s="4"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B27:B31 D5:H31">
-    <cfRule type="expression" dxfId="4" priority="96" stopIfTrue="1">
-      <formula>($F5="√")</formula>
+  <conditionalFormatting sqref="C5:C26">
+    <cfRule type="containsText" dxfId="4" priority="23" operator="containsText" text="LOW">
+      <formula>NOT(ISERROR(SEARCH("LOW",C5)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="3" priority="24" operator="containsText" text="MEDIUM">
+      <formula>NOT(ISERROR(SEARCH("MEDIUM",C5)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="2" priority="25" operator="containsText" text="HIGH">
+      <formula>NOT(ISERROR(SEARCH("HIGH",C5)))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="1" priority="98" stopIfTrue="1">
+      <formula>($F10="√")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C5:C26">
-    <cfRule type="containsText" dxfId="3" priority="23" operator="containsText" text="LOW">
-      <formula>NOT(ISERROR(SEARCH("LOW",C5)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="2" priority="24" operator="containsText" text="MEDIUM">
-      <formula>NOT(ISERROR(SEARCH("MEDIUM",C5)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="1" priority="25" operator="containsText" text="HIGH">
-      <formula>NOT(ISERROR(SEARCH("HIGH",C5)))</formula>
+  <conditionalFormatting sqref="D5:H31 B27:B31">
+    <cfRule type="expression" dxfId="0" priority="96" stopIfTrue="1">
+      <formula>($F5="√")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G5:G31">
@@ -1737,11 +1637,6 @@
           <x14:id>{46CB8FF5-0D6D-4783-B376-6ACC7FD916DC}</x14:id>
         </ext>
       </extLst>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C5:C26">
-    <cfRule type="expression" dxfId="0" priority="98" stopIfTrue="1">
-      <formula>($F10="√")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
@@ -1810,7 +1705,7 @@
           <x14:formula1>
             <xm:f>Sheet1!$A$2:$A$6</xm:f>
           </x14:formula1>
-          <xm:sqref>D5:D23</xm:sqref>
+          <xm:sqref>D5:D26</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>

<commit_message>
O, P, Q, R Complete but Untested
</commit_message>
<xml_diff>
--- a/UR5 Tasks.xlsx
+++ b/UR5 Tasks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ucliveac-my.sharepoint.com/personal/mcu55_uclive_ac_nz/Documents/4th Year/ENMT482/ENMT482-Robot-Coffee-Special/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="163" documentId="8_{5F62A8B3-761C-4507-BA16-EE4921CCE146}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7B0EBB06-80A5-4437-96C0-6BD21D058AD3}"/>
+  <xr:revisionPtr revIDLastSave="169" documentId="8_{5F62A8B3-761C-4507-BA16-EE4921CCE146}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A5A22F0B-9AF4-4D3F-B2BE-95024B477989}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="64">
   <si>
     <t>ACTION ITEMS</t>
   </si>
@@ -1170,8 +1170,8 @@
       <c r="F6" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="G6" s="14" t="s">
-        <v>63</v>
+      <c r="G6" s="14">
+        <v>1</v>
       </c>
       <c r="H6" s="4"/>
       <c r="J6" s="10"/>
@@ -1382,8 +1382,8 @@
         <v>61</v>
       </c>
       <c r="F17" s="23"/>
-      <c r="G17" s="14" t="s">
-        <v>10</v>
+      <c r="G17" s="14">
+        <v>1</v>
       </c>
       <c r="H17" s="4"/>
     </row>
@@ -1420,8 +1420,8 @@
         <v>62</v>
       </c>
       <c r="F19" s="23"/>
-      <c r="G19" s="14">
-        <v>0.5</v>
+      <c r="G19" s="14" t="s">
+        <v>63</v>
       </c>
       <c r="H19" s="4"/>
     </row>
@@ -1439,8 +1439,8 @@
         <v>62</v>
       </c>
       <c r="F20" s="23"/>
-      <c r="G20" s="14" t="s">
-        <v>10</v>
+      <c r="G20" s="14">
+        <v>0.75</v>
       </c>
       <c r="H20" s="4"/>
     </row>
@@ -1459,7 +1459,7 @@
       </c>
       <c r="F21" s="23"/>
       <c r="G21" s="14" t="s">
-        <v>10</v>
+        <v>63</v>
       </c>
       <c r="H21" s="15"/>
     </row>
@@ -1478,7 +1478,7 @@
       </c>
       <c r="F22" s="23"/>
       <c r="G22" s="14" t="s">
-        <v>10</v>
+        <v>63</v>
       </c>
       <c r="H22" s="4"/>
     </row>

</xml_diff>

<commit_message>
Part L, S, R, Q
</commit_message>
<xml_diff>
--- a/UR5 Tasks.xlsx
+++ b/UR5 Tasks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ucliveac-my.sharepoint.com/personal/mcu55_uclive_ac_nz/Documents/4th Year/ENMT482/ENMT482-Robot-Coffee-Special/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="169" documentId="8_{5F62A8B3-761C-4507-BA16-EE4921CCE146}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A5A22F0B-9AF4-4D3F-B2BE-95024B477989}"/>
+  <xr:revisionPtr revIDLastSave="172" documentId="8_{5F62A8B3-761C-4507-BA16-EE4921CCE146}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2A857787-9F07-436F-B59B-FF9FC3502DFB}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="64">
   <si>
     <t>ACTION ITEMS</t>
   </si>
@@ -1364,7 +1364,7 @@
       </c>
       <c r="F16" s="23"/>
       <c r="G16" s="14" t="s">
-        <v>10</v>
+        <v>63</v>
       </c>
       <c r="H16" s="4"/>
     </row>
@@ -1439,8 +1439,8 @@
         <v>62</v>
       </c>
       <c r="F20" s="23"/>
-      <c r="G20" s="14">
-        <v>0.75</v>
+      <c r="G20" s="14" t="s">
+        <v>63</v>
       </c>
       <c r="H20" s="4"/>
     </row>
@@ -1497,7 +1497,7 @@
       </c>
       <c r="F23" s="23"/>
       <c r="G23" s="14" t="s">
-        <v>10</v>
+        <v>63</v>
       </c>
       <c r="H23" s="15"/>
     </row>

</xml_diff>

<commit_message>
Completed Sections O through V (and L) -> Untested
</commit_message>
<xml_diff>
--- a/UR5 Tasks.xlsx
+++ b/UR5 Tasks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ucliveac-my.sharepoint.com/personal/mcu55_uclive_ac_nz/Documents/4th Year/ENMT482/ENMT482-Robot-Coffee-Special/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="172" documentId="8_{5F62A8B3-761C-4507-BA16-EE4921CCE146}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2A857787-9F07-436F-B59B-FF9FC3502DFB}"/>
+  <xr:revisionPtr revIDLastSave="175" documentId="8_{5F62A8B3-761C-4507-BA16-EE4921CCE146}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B0F086CD-9161-47F0-8893-BB9C2D5723D1}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1516,7 +1516,7 @@
       </c>
       <c r="F24" s="23"/>
       <c r="G24" s="14" t="s">
-        <v>10</v>
+        <v>63</v>
       </c>
       <c r="H24" s="15"/>
     </row>
@@ -1535,7 +1535,7 @@
       </c>
       <c r="F25" s="23"/>
       <c r="G25" s="14" t="s">
-        <v>10</v>
+        <v>63</v>
       </c>
       <c r="H25" s="15"/>
     </row>
@@ -1554,7 +1554,7 @@
       </c>
       <c r="F26" s="25"/>
       <c r="G26" s="14" t="s">
-        <v>10</v>
+        <v>63</v>
       </c>
       <c r="H26" s="4"/>
       <c r="J26"/>

</xml_diff>